<commit_message>
Import Applied seminars and update visitors
</commit_message>
<xml_diff>
--- a/outputs/01a0719b-f374-7590-b5ae-261ff64e352b/applied-economics-2026-27.xlsx
+++ b/outputs/01a0719b-f374-7590-b5ae-261ff64e352b/applied-economics-2026-27.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Seminars" sheetId="1" r:id="R50388166bf594f33"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Seminars" sheetId="1" r:id="Rd36e937883fb4aa9"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -72,13 +72,31 @@
       </x:patternFill>
     </x:fill>
   </x:fills>
-  <x:borders count="1">
+  <x:borders count="4">
     <x:border/>
+    <x:border>
+      <x:bottom style="thin">
+        <x:color rgb="FFD8DEE3"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:top style="thin">
+        <x:color rgb="FFD8DEE3"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFD8DEE3"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:top style="thin">
+        <x:color rgb="FFD8DEE3"/>
+      </x:top>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="16">
+  <x:cellXfs count="24">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -101,16 +119,40 @@
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="200" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="200" fontId="2" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="2" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -123,7 +165,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="applied_economics_seminars" displayName="applied_economics_seminars" ref="A1:J2" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="applied_economics_seminars" displayName="applied_economics_seminars" ref="A1:J21" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="10">
     <x:tableColumn id="1" name="Date"/>
     <x:tableColumn id="2" name="Speaker"/>
@@ -380,34 +422,390 @@
       </x:c>
     </x:row>
     <x:row r="2" ht="15" hidden="0" customHeight="1">
-      <x:c r="A2" s="12" t="str"/>
-      <x:c r="B2" s="13" t="str"/>
-      <x:c r="C2" s="13" t="str"/>
-      <x:c r="D2" s="13" t="str"/>
-      <x:c r="E2" s="13" t="str"/>
-      <x:c r="F2" s="13" t="str"/>
-      <x:c r="G2" s="13" t="str"/>
-      <x:c r="H2" s="11" t="str"/>
-      <x:c r="I2" s="11" t="str"/>
-      <x:c r="J2" s="11" t="str"/>
-    </x:row>
-    <x:row r="4">
-      <x:c r="A4" s="14" t="str">
+      <x:c r="A2" s="13" t="n">
+        <x:v>46294</x:v>
+      </x:c>
+      <x:c r="B2" s="10" t="str">
+        <x:v>Andrew Garin</x:v>
+      </x:c>
+      <x:c r="C2" s="19" t="str"/>
+      <x:c r="D2" s="19" t="str"/>
+      <x:c r="E2" s="19" t="str"/>
+      <x:c r="F2" s="19" t="str"/>
+      <x:c r="G2" s="10" t="str">
+        <x:v>Scheduled</x:v>
+      </x:c>
+      <x:c r="H2" s="16" t="str"/>
+      <x:c r="I2" s="16" t="str"/>
+      <x:c r="J2" s="16" t="str"/>
+    </x:row>
+    <x:row r="3" ht="15" hidden="0" customHeight="1">
+      <x:c r="A3" s="14" t="n">
+        <x:v>46301</x:v>
+      </x:c>
+      <x:c r="B3" s="11" t="str">
+        <x:v>Mitsuru Igami</x:v>
+      </x:c>
+      <x:c r="C3" s="20" t="str"/>
+      <x:c r="D3" s="20" t="str"/>
+      <x:c r="E3" s="20" t="str"/>
+      <x:c r="F3" s="20" t="str"/>
+      <x:c r="G3" s="11" t="str">
+        <x:v>Scheduled</x:v>
+      </x:c>
+      <x:c r="H3" s="17" t="str"/>
+      <x:c r="I3" s="17" t="str"/>
+      <x:c r="J3" s="17" t="str"/>
+    </x:row>
+    <x:row r="4" ht="15" hidden="0" customHeight="1">
+      <x:c r="A4" s="14" t="n">
+        <x:v>46308</x:v>
+      </x:c>
+      <x:c r="B4" s="11" t="str">
+        <x:v>Chris Neilson</x:v>
+      </x:c>
+      <x:c r="C4" s="20" t="str"/>
+      <x:c r="D4" s="20" t="str"/>
+      <x:c r="E4" s="20" t="str"/>
+      <x:c r="F4" s="20" t="str"/>
+      <x:c r="G4" s="11" t="str">
+        <x:v>Scheduled</x:v>
+      </x:c>
+      <x:c r="H4" s="17" t="str"/>
+      <x:c r="I4" s="17" t="str"/>
+      <x:c r="J4" s="17" t="str"/>
+    </x:row>
+    <x:row r="5" ht="15" hidden="0" customHeight="1">
+      <x:c r="A5" s="14" t="n">
+        <x:v>46315</x:v>
+      </x:c>
+      <x:c r="B5" s="11" t="str">
+        <x:v>Melanie Morten</x:v>
+      </x:c>
+      <x:c r="C5" s="20" t="str"/>
+      <x:c r="D5" s="20" t="str"/>
+      <x:c r="E5" s="20" t="str"/>
+      <x:c r="F5" s="20" t="str"/>
+      <x:c r="G5" s="11" t="str">
+        <x:v>Cancelled</x:v>
+      </x:c>
+      <x:c r="H5" s="17" t="str"/>
+      <x:c r="I5" s="17" t="str"/>
+      <x:c r="J5" s="17" t="str"/>
+    </x:row>
+    <x:row r="6" ht="15" hidden="0" customHeight="1">
+      <x:c r="A6" s="14" t="n">
+        <x:v>46321</x:v>
+      </x:c>
+      <x:c r="B6" s="11" t="str">
+        <x:v>Lawrence Schmidt</x:v>
+      </x:c>
+      <x:c r="C6" s="20" t="str"/>
+      <x:c r="D6" s="20" t="str"/>
+      <x:c r="E6" s="20" t="str"/>
+      <x:c r="F6" s="20" t="str"/>
+      <x:c r="G6" s="11" t="str">
+        <x:v>Scheduled</x:v>
+      </x:c>
+      <x:c r="H6" s="17" t="str"/>
+      <x:c r="I6" s="17" t="str"/>
+      <x:c r="J6" s="17" t="str"/>
+    </x:row>
+    <x:row r="7" ht="15" hidden="0" customHeight="1">
+      <x:c r="A7" s="14" t="n">
+        <x:v>46329</x:v>
+      </x:c>
+      <x:c r="B7" s="11" t="str">
+        <x:v>Benjamin M. Scuderi</x:v>
+      </x:c>
+      <x:c r="C7" s="20" t="str"/>
+      <x:c r="D7" s="20" t="str"/>
+      <x:c r="E7" s="20" t="str"/>
+      <x:c r="F7" s="20" t="str"/>
+      <x:c r="G7" s="11" t="str">
+        <x:v>Scheduled</x:v>
+      </x:c>
+      <x:c r="H7" s="17" t="str"/>
+      <x:c r="I7" s="17" t="str"/>
+      <x:c r="J7" s="17" t="str"/>
+    </x:row>
+    <x:row r="8" ht="15" hidden="0" customHeight="1">
+      <x:c r="A8" s="14" t="n">
+        <x:v>46357</x:v>
+      </x:c>
+      <x:c r="B8" s="11" t="str">
+        <x:v>Sebastian Otero</x:v>
+      </x:c>
+      <x:c r="C8" s="20" t="str"/>
+      <x:c r="D8" s="20" t="str"/>
+      <x:c r="E8" s="20" t="str"/>
+      <x:c r="F8" s="20" t="str"/>
+      <x:c r="G8" s="11" t="str">
+        <x:v>Scheduled</x:v>
+      </x:c>
+      <x:c r="H8" s="17" t="str"/>
+      <x:c r="I8" s="17" t="str"/>
+      <x:c r="J8" s="17" t="str"/>
+    </x:row>
+    <x:row r="9" ht="15" hidden="0" customHeight="1">
+      <x:c r="A9" s="14" t="n">
+        <x:v>46364</x:v>
+      </x:c>
+      <x:c r="B9" s="11" t="str">
+        <x:v>Tatiana Mocanu</x:v>
+      </x:c>
+      <x:c r="C9" s="20" t="str"/>
+      <x:c r="D9" s="20" t="str"/>
+      <x:c r="E9" s="20" t="str"/>
+      <x:c r="F9" s="20" t="str"/>
+      <x:c r="G9" s="11" t="str">
+        <x:v>Scheduled</x:v>
+      </x:c>
+      <x:c r="H9" s="17" t="str"/>
+      <x:c r="I9" s="17" t="str"/>
+      <x:c r="J9" s="17" t="str"/>
+    </x:row>
+    <x:row r="10" ht="15" hidden="0" customHeight="1">
+      <x:c r="A10" s="14" t="n">
+        <x:v>46370</x:v>
+      </x:c>
+      <x:c r="B10" s="11" t="str">
+        <x:v>Elena Simintzi</x:v>
+      </x:c>
+      <x:c r="C10" s="20" t="str"/>
+      <x:c r="D10" s="20" t="str"/>
+      <x:c r="E10" s="20" t="str"/>
+      <x:c r="F10" s="20" t="str"/>
+      <x:c r="G10" s="11" t="str">
+        <x:v>Scheduled</x:v>
+      </x:c>
+      <x:c r="H10" s="17" t="str"/>
+      <x:c r="I10" s="17" t="str"/>
+      <x:c r="J10" s="17" t="str"/>
+    </x:row>
+    <x:row r="11" ht="15" hidden="0" customHeight="1">
+      <x:c r="A11" s="14" t="n">
+        <x:v>46441</x:v>
+      </x:c>
+      <x:c r="B11" s="11" t="str">
+        <x:v>Enrico Moretti</x:v>
+      </x:c>
+      <x:c r="C11" s="20" t="str"/>
+      <x:c r="D11" s="20" t="str"/>
+      <x:c r="E11" s="20" t="str"/>
+      <x:c r="F11" s="20" t="str"/>
+      <x:c r="G11" s="11" t="str">
+        <x:v>Scheduled</x:v>
+      </x:c>
+      <x:c r="H11" s="17" t="str"/>
+      <x:c r="I11" s="17" t="str"/>
+      <x:c r="J11" s="17" t="str"/>
+    </x:row>
+    <x:row r="12" ht="15" hidden="0" customHeight="1">
+      <x:c r="A12" s="14" t="n">
+        <x:v>46448</x:v>
+      </x:c>
+      <x:c r="B12" s="11" t="str">
+        <x:v>Amanda Starc</x:v>
+      </x:c>
+      <x:c r="C12" s="20" t="str"/>
+      <x:c r="D12" s="20" t="str"/>
+      <x:c r="E12" s="20" t="str"/>
+      <x:c r="F12" s="20" t="str"/>
+      <x:c r="G12" s="11" t="str">
+        <x:v>Scheduled</x:v>
+      </x:c>
+      <x:c r="H12" s="17" t="str"/>
+      <x:c r="I12" s="17" t="str"/>
+      <x:c r="J12" s="17" t="str"/>
+    </x:row>
+    <x:row r="13" ht="15" hidden="0" customHeight="1">
+      <x:c r="A13" s="14" t="n">
+        <x:v>46455</x:v>
+      </x:c>
+      <x:c r="B13" s="11" t="str">
+        <x:v>Mathilde Munoz</x:v>
+      </x:c>
+      <x:c r="C13" s="20" t="str"/>
+      <x:c r="D13" s="20" t="str"/>
+      <x:c r="E13" s="20" t="str"/>
+      <x:c r="F13" s="20" t="str"/>
+      <x:c r="G13" s="11" t="str">
+        <x:v>Scheduled</x:v>
+      </x:c>
+      <x:c r="H13" s="17" t="str"/>
+      <x:c r="I13" s="17" t="str"/>
+      <x:c r="J13" s="17" t="str"/>
+    </x:row>
+    <x:row r="14" ht="15" hidden="0" customHeight="1">
+      <x:c r="A14" s="14" t="n">
+        <x:v>46462</x:v>
+      </x:c>
+      <x:c r="B14" s="11" t="str">
+        <x:v>Andrei Levchenko</x:v>
+      </x:c>
+      <x:c r="C14" s="20" t="str"/>
+      <x:c r="D14" s="20" t="str"/>
+      <x:c r="E14" s="20" t="str"/>
+      <x:c r="F14" s="20" t="str"/>
+      <x:c r="G14" s="11" t="str">
+        <x:v>Scheduled</x:v>
+      </x:c>
+      <x:c r="H14" s="17" t="str"/>
+      <x:c r="I14" s="17" t="str"/>
+      <x:c r="J14" s="17" t="str"/>
+    </x:row>
+    <x:row r="15" ht="15" hidden="0" customHeight="1">
+      <x:c r="A15" s="14" t="n">
+        <x:v>46467</x:v>
+      </x:c>
+      <x:c r="B15" s="11" t="str">
+        <x:v>Paul Goldsmith-Pinkham</x:v>
+      </x:c>
+      <x:c r="C15" s="20" t="str"/>
+      <x:c r="D15" s="20" t="str"/>
+      <x:c r="E15" s="20" t="str"/>
+      <x:c r="F15" s="20" t="str"/>
+      <x:c r="G15" s="11" t="str">
+        <x:v>Scheduled</x:v>
+      </x:c>
+      <x:c r="H15" s="17" t="str"/>
+      <x:c r="I15" s="17" t="str"/>
+      <x:c r="J15" s="17" t="str"/>
+    </x:row>
+    <x:row r="16" ht="15" hidden="0" customHeight="1">
+      <x:c r="A16" s="14" t="n">
+        <x:v>46504</x:v>
+      </x:c>
+      <x:c r="B16" s="11" t="str">
+        <x:v>Pedro Sant'Anna</x:v>
+      </x:c>
+      <x:c r="C16" s="20" t="str"/>
+      <x:c r="D16" s="20" t="str"/>
+      <x:c r="E16" s="20" t="str"/>
+      <x:c r="F16" s="20" t="str"/>
+      <x:c r="G16" s="11" t="str">
+        <x:v>Cancelled</x:v>
+      </x:c>
+      <x:c r="H16" s="17" t="str"/>
+      <x:c r="I16" s="17" t="str"/>
+      <x:c r="J16" s="17" t="str"/>
+    </x:row>
+    <x:row r="17" ht="15" hidden="0" customHeight="1">
+      <x:c r="A17" s="14" t="n">
+        <x:v>46511</x:v>
+      </x:c>
+      <x:c r="B17" s="11" t="str">
+        <x:v>Lance Lochner</x:v>
+      </x:c>
+      <x:c r="C17" s="20" t="str"/>
+      <x:c r="D17" s="20" t="str"/>
+      <x:c r="E17" s="20" t="str"/>
+      <x:c r="F17" s="20" t="str"/>
+      <x:c r="G17" s="11" t="str">
+        <x:v>Scheduled</x:v>
+      </x:c>
+      <x:c r="H17" s="17" t="str"/>
+      <x:c r="I17" s="17" t="str"/>
+      <x:c r="J17" s="17" t="str"/>
+    </x:row>
+    <x:row r="18" ht="15" hidden="0" customHeight="1">
+      <x:c r="A18" s="14" t="n">
+        <x:v>46518</x:v>
+      </x:c>
+      <x:c r="B18" s="11" t="str">
+        <x:v>Emily Breza</x:v>
+      </x:c>
+      <x:c r="C18" s="20" t="str"/>
+      <x:c r="D18" s="20" t="str"/>
+      <x:c r="E18" s="20" t="str"/>
+      <x:c r="F18" s="20" t="str"/>
+      <x:c r="G18" s="11" t="str">
+        <x:v>Scheduled</x:v>
+      </x:c>
+      <x:c r="H18" s="17" t="str"/>
+      <x:c r="I18" s="17" t="str"/>
+      <x:c r="J18" s="17" t="str"/>
+    </x:row>
+    <x:row r="19" ht="15" hidden="0" customHeight="1">
+      <x:c r="A19" s="14" t="n">
+        <x:v>46525</x:v>
+      </x:c>
+      <x:c r="B19" s="11" t="str">
+        <x:v>Florian Ederer</x:v>
+      </x:c>
+      <x:c r="C19" s="20" t="str"/>
+      <x:c r="D19" s="20" t="str"/>
+      <x:c r="E19" s="20" t="str"/>
+      <x:c r="F19" s="20" t="str"/>
+      <x:c r="G19" s="11" t="str">
+        <x:v>Scheduled</x:v>
+      </x:c>
+      <x:c r="H19" s="17" t="str"/>
+      <x:c r="I19" s="17" t="str"/>
+      <x:c r="J19" s="17" t="str"/>
+    </x:row>
+    <x:row r="20" ht="15" hidden="0" customHeight="1">
+      <x:c r="A20" s="14" t="n">
+        <x:v>46532</x:v>
+      </x:c>
+      <x:c r="B20" s="11" t="str">
+        <x:v>Oriana Bandiera</x:v>
+      </x:c>
+      <x:c r="C20" s="20" t="str"/>
+      <x:c r="D20" s="20" t="str"/>
+      <x:c r="E20" s="20" t="str"/>
+      <x:c r="F20" s="20" t="str"/>
+      <x:c r="G20" s="11" t="str">
+        <x:v>Scheduled</x:v>
+      </x:c>
+      <x:c r="H20" s="17" t="str"/>
+      <x:c r="I20" s="17" t="str"/>
+      <x:c r="J20" s="17" t="str"/>
+    </x:row>
+    <x:row r="21" ht="15" hidden="0" customHeight="1">
+      <x:c r="A21" s="15" t="n">
+        <x:v>46539</x:v>
+      </x:c>
+      <x:c r="B21" s="12" t="str">
+        <x:v>Chinhui Juhn</x:v>
+      </x:c>
+      <x:c r="C21" s="21" t="str"/>
+      <x:c r="D21" s="21" t="str"/>
+      <x:c r="E21" s="21" t="str"/>
+      <x:c r="F21" s="21" t="str"/>
+      <x:c r="G21" s="12" t="str">
+        <x:v>Scheduled</x:v>
+      </x:c>
+      <x:c r="H21" s="18" t="str"/>
+      <x:c r="I21" s="18" t="str"/>
+      <x:c r="J21" s="18" t="str"/>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="22" t="str">
         <x:v>Overrides</x:v>
       </x:c>
-      <x:c r="B4" s="15" t="str">
+      <x:c r="B23" s="23" t="str">
         <x:v>Blue columns are optional. A gold value replaces the series default for that seminar.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="22" t="str">
+        <x:v>Source</x:v>
+      </x:c>
+      <x:c r="B24" s="23" t="str">
+        <x:v>https://docs.google.com/spreadsheets/d/1dBRaQ5umcfPDVclwKMPpc2sKSEDHaTf5/edit?gid=647007165</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:dataValidations count="1">
-    <x:dataValidation type="list" sqref="G2">
+    <x:dataValidation type="list" sqref="G2:G21">
       <x:formula1>"Scheduled,JMC,Cancelled,Postponed,TBA"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb65531133e094c34"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Red5bce9ee2af4e39"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>